<commit_message>
refactor: add config files, Fe constraint, FeO->Fe conversion, and clean optimizer code
</commit_message>
<xml_diff>
--- a/assets/BF02_Ores_Chemical_Composition.xlsx
+++ b/assets/BF02_Ores_Chemical_Composition.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,11 +46,6 @@
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -100,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -120,8 +115,6 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -487,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M22"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -508,7 +501,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BF-02 BUNKER - ORES AVERAGE CHEMICAL COMPOSITION (2025-26)</t>
+          <t>BF-02 BUNKER - ORES MONTHLY CHEMICAL COMPOSITION</t>
         </is>
       </c>
     </row>
@@ -587,7 +580,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>63.818</v>
+        <v>64.965</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -595,34 +588,34 @@
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>1.85</v>
+        <v>3.657</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>1.101</v>
+        <v>0.903</v>
       </c>
       <c r="F4" s="4" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="J4" s="4" t="n">
         <v>0.029</v>
       </c>
-      <c r="G4" s="4" t="n">
-        <v>0.041</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>0.027</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>0.021</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>0.041</v>
-      </c>
       <c r="K4" s="4" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.049</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>0.047</v>
+        <v>0.068</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>2.008</v>
+        <v>1.832</v>
       </c>
     </row>
     <row r="5">
@@ -632,7 +625,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>54.205</v>
+        <v>55.695</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
@@ -640,34 +633,34 @@
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>14.402</v>
+        <v>13.27</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>2.2</v>
+        <v>3.28</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>0.029</v>
+        <v>0.031</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.093</v>
+        <v>0.141</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>0.026</v>
+        <v>0.022</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>0.02</v>
+        <v>0.034</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>0.047</v>
+        <v>0.062</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>0.058</v>
+        <v>0.038</v>
       </c>
       <c r="L5" s="4" t="n">
-        <v>0.045</v>
+        <v>0.062</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>2.075</v>
+        <v>2.67</v>
       </c>
     </row>
     <row r="6">
@@ -677,7 +670,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>54.858</v>
+        <v>62.66</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
@@ -685,34 +678,34 @@
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>1.159</v>
+        <v>1.298</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>2.062</v>
+        <v>2.332</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>0.038</v>
+        <v>0.042</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.179</v>
+        <v>0.202</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>0.016</v>
+        <v>0.017</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>0.013</v>
+        <v>0.014</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>0.027</v>
+        <v>0.028</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>0.058</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>0.048</v>
+        <v>0.046</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>5.255</v>
+        <v>5.98</v>
       </c>
     </row>
     <row r="7">
@@ -722,7 +715,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>61.324</v>
+        <v>64.04000000000001</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
@@ -730,34 +723,34 @@
         </is>
       </c>
       <c r="D7" s="4" t="n">
-        <v>4.745</v>
+        <v>4.191</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>2.118</v>
+        <v>1.937</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>0.045</v>
+        <v>0.047</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.103</v>
+        <v>0.116</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>0.036</v>
+        <v>0.038</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>0.041</v>
+        <v>0.03</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>0.042</v>
+        <v>0.026</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>0.725</v>
+        <v>1.1</v>
       </c>
       <c r="L7" s="4" t="n">
-        <v>0.114</v>
+        <v>0.21</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>0.465</v>
+        <v>0.503</v>
       </c>
     </row>
     <row r="8">
@@ -767,7 +760,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>61.637</v>
+        <v>62.783</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
@@ -775,34 +768,34 @@
         </is>
       </c>
       <c r="D8" s="4" t="n">
-        <v>3.132</v>
+        <v>4.893</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>3.459</v>
+        <v>2.206</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>0.047</v>
+        <v>0.045</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>0.176</v>
+        <v>0.094</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>0.012</v>
+        <v>0.035</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>0.028</v>
+        <v>0.024</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>0.034</v>
+        <v>0.027</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>0.068</v>
+        <v>0.082</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>0.061</v>
+        <v>0.052</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>2.662</v>
+        <v>2.626</v>
       </c>
     </row>
     <row r="9">
@@ -812,7 +805,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>61.624</v>
+        <v>62.787</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
@@ -820,34 +813,34 @@
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>3.126</v>
+        <v>4.875</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>3.461</v>
+        <v>2.214</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>0.047</v>
+        <v>0.045</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.176</v>
+        <v>0.096</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>0.012</v>
+        <v>0.036</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>0.028</v>
+        <v>0.024</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>0.034</v>
+        <v>0.027</v>
       </c>
       <c r="K9" s="4" t="n">
-        <v>0.067</v>
+        <v>0.083</v>
       </c>
       <c r="L9" s="4" t="n">
-        <v>0.061</v>
+        <v>0.053</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>2.662</v>
+        <v>2.637</v>
       </c>
     </row>
     <row r="10">
@@ -857,7 +850,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>55.658</v>
+        <v>57.288</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
@@ -865,34 +858,34 @@
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>4.838</v>
+        <v>4.314</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>5.297</v>
+        <v>6.019</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>0.041</v>
+        <v>0.044</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.277</v>
+        <v>0.32</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>0.02</v>
+        <v>0.011</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>0.03</v>
+        <v>0.034</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>0.06</v>
+        <v>0.076</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>0.173</v>
+        <v>0.157</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>0.08</v>
+        <v>0.073</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>6.178</v>
+        <v>6.536</v>
       </c>
     </row>
     <row r="11">
@@ -902,7 +895,7 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>50.694</v>
+        <v>58.987</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
@@ -910,34 +903,34 @@
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>2.007</v>
+        <v>2.255</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>4.173</v>
+        <v>4.825</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>0.067</v>
+        <v>0.077</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>0.188</v>
+        <v>0.208</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.008</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>0.027</v>
+        <v>0.03</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>0.049</v>
+        <v>0.055</v>
       </c>
       <c r="K11" s="4" t="n">
-        <v>0.042</v>
+        <v>0.035</v>
       </c>
       <c r="L11" s="4" t="n">
-        <v>0.027</v>
+        <v>0.022</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>6.569</v>
+        <v>7.593</v>
       </c>
     </row>
     <row r="12">
@@ -947,7 +940,7 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>52.473</v>
+        <v>56.781</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
@@ -955,34 +948,34 @@
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>6.424</v>
+        <v>6.861</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>2.111</v>
+        <v>2.2</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>0.104</v>
+        <v>0.112</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.064</v>
+        <v>0.066</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>0.033</v>
+        <v>0.028</v>
       </c>
       <c r="I12" s="4" t="n">
         <v>0.036</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>0.241</v>
+        <v>0.235</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>0.456</v>
+        <v>0.465</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>0.057</v>
+        <v>0.058</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>7.354</v>
+        <v>7.887</v>
       </c>
     </row>
     <row r="13">
@@ -992,7 +985,7 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>42.659</v>
+        <v>49.687</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
@@ -1000,34 +993,34 @@
         </is>
       </c>
       <c r="D13" s="4" t="n">
-        <v>5.602</v>
+        <v>6.523</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>3.37</v>
+        <v>3.93</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>0.028</v>
+        <v>0.032</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>12.191</v>
+        <v>14.203</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>0.034</v>
+        <v>0.039</v>
       </c>
       <c r="I13" s="4" t="n">
-        <v>0.04</v>
+        <v>0.046</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>0.254</v>
+        <v>0.293</v>
       </c>
       <c r="K13" s="4" t="n">
-        <v>0.257</v>
+        <v>0.3</v>
       </c>
       <c r="L13" s="4" t="n">
-        <v>0.63</v>
+        <v>0.733</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>1.412</v>
+        <v>1.617</v>
       </c>
     </row>
     <row r="14">
@@ -1037,7 +1030,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>49.584</v>
+        <v>51.408</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
@@ -1045,34 +1038,34 @@
         </is>
       </c>
       <c r="D14" s="4" t="n">
-        <v>9.193</v>
+        <v>10.126</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>7.59</v>
+        <v>7.488</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>0.185</v>
+        <v>0.121</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.784</v>
+        <v>0.779</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>0.027</v>
+        <v>0.029</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>0.02</v>
+        <v>0.034</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>0.145</v>
+        <v>0.125</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>0.137</v>
+        <v>0.156</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>0.098</v>
+        <v>0.111</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>8.519</v>
+        <v>7.252</v>
       </c>
     </row>
     <row r="15">
@@ -1082,7 +1075,7 @@
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>27.06</v>
+        <v>30.66</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
@@ -1090,34 +1083,34 @@
         </is>
       </c>
       <c r="D15" s="4" t="n">
-        <v>3.1</v>
+        <v>3.57</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>5.463</v>
+        <v>6.05</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0.028</v>
+        <v>0.024</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.206</v>
+        <v>0.261</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>0.039</v>
+        <v>0.04</v>
       </c>
       <c r="I15" s="4" t="n">
-        <v>0.499</v>
+        <v>0.457</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>22.14</v>
+        <v>22.87</v>
       </c>
       <c r="K15" s="4" t="n">
-        <v>0.413</v>
+        <v>0.7</v>
       </c>
       <c r="L15" s="4" t="n">
-        <v>0.075</v>
+        <v>0.1</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>10.265</v>
+        <v>11.49</v>
       </c>
     </row>
     <row r="16">
@@ -1127,37 +1120,37 @@
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>54.409</v>
+        <v>54.984</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>9.246</v>
+        <v>9.061999999999999</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>5.437</v>
+        <v>5.382</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>2.345</v>
+        <v>2.43</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>0.062</v>
+        <v>0.048</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.181</v>
+        <v>0.151</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>0.053</v>
+        <v>0.033</v>
       </c>
       <c r="I16" s="4" t="n">
-        <v>0.067</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>0.258</v>
+        <v>0.156</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>10.603</v>
+        <v>10.773</v>
       </c>
       <c r="L16" s="4" t="n">
-        <v>1.844</v>
+        <v>1.947</v>
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
@@ -1165,48 +1158,9 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>Notes:</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="8" t="inlineStr">
-        <is>
-          <t>Acore Industries is a Mn ore (high %MnO ~22%), not a typical iron ore.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t>Titani Ferrous CLO has very high %TiO2 (~12%) - titaniferous iron ore.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t>%FeO is available only for Sinter. Other ores report %Fe(T) only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>All values are averages computed from available sample data in BF-02 Bunker 2025-26.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A21:H21"/>
+  <mergeCells count="1">
     <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A20:H20"/>
-    <mergeCell ref="A19:H19"/>
-    <mergeCell ref="A22:H22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>